<commit_message>
Clean public source locators without changing academic facts; enforce metadata guard and versioned historical contracts
</commit_message>
<xml_diff>
--- a/site/exports/csu-physics.xlsx
+++ b/site/exports/csu-physics.xlsx
@@ -2854,7 +2854,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Junwei Fu", "source_url": "https://faculty.csu.edu.cn/~m2INBz/zh_CN/index.htm", "source_locator": "L79"}</t>
+          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Junwei Fu", "source_url": "https://faculty.csu.edu.cn/~m2INBz/zh_CN/index.htm", "source_locator": "个人主页中题名《Theoretical Insights into the Selectivity of Single-Atom Fe–N–C Catalysts for Electrochemical NOx Reduction》的书目条目"}</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Junwei Fu", "source_url": "https://faculty.csu.edu.cn/~m2INBz/zh_CN/index.htm", "source_locator": "L80"}</t>
+          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Junwei Fu", "source_url": "https://faculty.csu.edu.cn/~m2INBz/zh_CN/index.htm", "source_locator": "个人主页中题名《Sustainable conversion of alkaline nitrate to ammonia at activities greater than 2 A cm-2》的书目条目"}</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Ai-Min Guo", "source_url": "https://faculty.csu.edu.cn/guoaimin/zh_CN/index.htm", "source_locator": "L60"}</t>
+          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Ai-Min Guo", "source_url": "https://faculty.csu.edu.cn/guoaimin/zh_CN/index.htm", "source_locator": "个人主页中题名《Spin-to-charge conversion driven by inverse chiral-induced spin selectivity》的书目条目"}</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Ai-Min Guo", "source_url": "https://faculty.csu.edu.cn/guoaimin/zh_CN/index.htm", "source_locator": "L61"}</t>
+          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Ai-Min Guo", "source_url": "https://faculty.csu.edu.cn/guoaimin/zh_CN/index.htm", "source_locator": "个人主页中题名《Spin-driven Enantioselective Regulation of Cyclooxygenase-2 Activity for Rheumatoid Arthritis Therapy via Chiral Gold Nanohelices》的书目条目"}</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Guang-hua Guo", "source_url": "https://faculty.csu.edu.cn/guoguanghua/zh_CN/index.htm", "source_locator": "L71"}</t>
+          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Guang-hua Guo", "source_url": "https://faculty.csu.edu.cn/guoguanghua/zh_CN/index.htm", "source_locator": "个人主页中题名《Manipulation of the polarized magnon transmission in trilayer magnonic spin-valve》的书目条目"}</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Guang-hua Guo", "source_url": "https://faculty.csu.edu.cn/guoguanghua/zh_CN/index.htm", "source_locator": "L73"}</t>
+          <t>{"status": "listed_in_official_personal_bibliography", "matched_author": "Guang-hua Guo", "source_url": "https://faculty.csu.edu.cn/guoguanghua/zh_CN/index.htm", "source_locator": "个人主页中题名《Reconfigurable Spin-wave Coupler Based on Domain Wall Channels》的书目条目"}</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">

</xml_diff>